<commit_message>
dd-screener: merge 6/4 supplement (29 tickers) → coverage 194→223/225
- Merged DD_universe_EPS_supplement_20260604.xlsx (30 rows, 3443 overlap kept
  from main) into the 6/4 main Excel via surgical XML append (preserves Koyfin
  shared-string structure; openpyxl rewrite uses inlineStr which the raw-XML
  loader can't read → 0 coverage, avoided).
- Adds previously-uncovered US/ADR + TW names: UNH/MRK/ABBV/GILD/MCK/COF/CAH/
  COR/EHC/J/LEU/MP/NUE/RACE/RIO/SOFI/TMDX/TPC/VALE/BHP/ESLT/RKLB/SU.FR/ABB +
  TW 2327/2345/2368/3653/5274 — all now eps_source=xlsx.
- 未覆蓋 31→2 (LYC.AX/VACN.SW only); 缺漏紅字 24→0.
- GILD/ESLT/RKLB negatives/blanks → CAGR None (handled). FX applied to TW.
- NVDA/AVGO unchanged (no regression). Baseline 2026-05.json intact.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/eps-estimates/DD_universe_EPS_estimates_20260604.xlsx
+++ b/data/eps-estimates/DD_universe_EPS_estimates_20260604.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
   <si>
     <t xml:space="preserve">Ticker</t>
   </si>
@@ -705,6 +705,93 @@
   </si>
   <si>
     <t xml:space="preserve">FY1→FY2 = (FY2-FY1)/|FY1|; FY1→FY3 CAGR = (FY3/FY1)^0.5 - 1 (valid only when both positive)</t>
+  </si>
+  <si>
+    <t>2327</t>
+  </si>
+  <si>
+    <t>2345</t>
+  </si>
+  <si>
+    <t>2368</t>
+  </si>
+  <si>
+    <t>3653</t>
+  </si>
+  <si>
+    <t>5274</t>
+  </si>
+  <si>
+    <t>ABB</t>
+  </si>
+  <si>
+    <t>ABBV</t>
+  </si>
+  <si>
+    <t>BHP</t>
+  </si>
+  <si>
+    <t>CAH</t>
+  </si>
+  <si>
+    <t>COF</t>
+  </si>
+  <si>
+    <t>COR</t>
+  </si>
+  <si>
+    <t>EHC</t>
+  </si>
+  <si>
+    <t>ESLT</t>
+  </si>
+  <si>
+    <t>GILD</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>LEU</t>
+  </si>
+  <si>
+    <t>MCK</t>
+  </si>
+  <si>
+    <t>MP</t>
+  </si>
+  <si>
+    <t>MRK</t>
+  </si>
+  <si>
+    <t>NUE</t>
+  </si>
+  <si>
+    <t>RACE</t>
+  </si>
+  <si>
+    <t>RIO</t>
+  </si>
+  <si>
+    <t>RKLB</t>
+  </si>
+  <si>
+    <t>SOFI</t>
+  </si>
+  <si>
+    <t>SU.FR</t>
+  </si>
+  <si>
+    <t>TMDX</t>
+  </si>
+  <si>
+    <t>TPC</t>
+  </si>
+  <si>
+    <t>UNH</t>
+  </si>
+  <si>
+    <t>VALE</t>
   </si>
 </sst>
 </file>
@@ -2582,7 +2669,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G197"/>
+  <dimension ref="A1:G226"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -7691,8 +7778,660 @@
         <v>0.129120936546249</v>
       </c>
     </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B198" s="3" t="n">
+        <v>0.56</v>
+      </c>
+      <c r="C198" s="3" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="D198" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E198" s="4" t="n">
+        <v>0.357142857142857</v>
+      </c>
+      <c r="F198" s="4" t="n">
+        <v>0.355263157894737</v>
+      </c>
+      <c r="G198" s="4" t="n">
+        <v>0.356202681860538</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B199" s="3" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="C199" s="3" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="D199" s="3" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="E199" s="4" t="n">
+        <v>0.254980079681275</v>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>0.40952380952381</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>0.330009136355403</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B200" s="3" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="C200" s="3" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="D200" s="3" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E200" s="4" t="n">
+        <v>0.723214285714286</v>
+      </c>
+      <c r="F200" s="4" t="n">
+        <v>0.492227979274611</v>
+      </c>
+      <c r="G200" s="4" t="n">
+        <v>0.603567451474546</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B201" s="3" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="C201" s="3" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="D201" s="3" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E201" s="4" t="n">
+        <v>1.04945054945055</v>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>0.554959785522788</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>0.785164750607962</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B202" s="3" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="C202" s="3" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="D202" s="3" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="E202" s="4" t="n">
+        <v>0.47275641025641</v>
+      </c>
+      <c r="F202" s="4" t="n">
+        <v>0.612622415669206</v>
+      </c>
+      <c r="G202" s="4" t="n">
+        <v>0.541103500742244</v>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B203" s="3" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="C203" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D203" s="3" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="E203" s="4" t="n">
+        <v>0.0862619808306709</v>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>0.0970588235294118</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>0.0916470541044043</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B204" s="3" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="C204" s="3" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="D204" s="3" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="E204" s="4" t="n">
+        <v>0.141052631578947</v>
+      </c>
+      <c r="F204" s="4" t="n">
+        <v>0.100246002460025</v>
+      </c>
+      <c r="G204" s="4" t="n">
+        <v>0.120463563214453</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B205" s="3" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="C205" s="3" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="D205" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="E205" s="4" t="n">
+        <v>0.00392156862745107</v>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>-0.0390625</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>-0.0178055781297976</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B206" s="3" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="C206" s="3" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="D206" s="3" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="E206" s="4" t="n">
+        <v>0.112349117920149</v>
+      </c>
+      <c r="F206" s="4" t="n">
+        <v>0.128547579298831</v>
+      </c>
+      <c r="G206" s="4" t="n">
+        <v>0.120419075330287</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B207" s="3" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="C207" s="3" t="n">
+        <v>24.29</v>
+      </c>
+      <c r="D207" s="3" t="n">
+        <v>28.54</v>
+      </c>
+      <c r="E207" s="4" t="n">
+        <v>0.232994923857868</v>
+      </c>
+      <c r="F207" s="4" t="n">
+        <v>0.174969123095924</v>
+      </c>
+      <c r="G207" s="4" t="n">
+        <v>0.203632404211105</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B208" s="3" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="C208" s="3" t="n">
+        <v>19.78</v>
+      </c>
+      <c r="D208" s="3" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E208" s="4" t="n">
+        <v>0.114366197183099</v>
+      </c>
+      <c r="F208" s="4" t="n">
+        <v>0.107178968655207</v>
+      </c>
+      <c r="G208" s="4" t="n">
+        <v>0.110766769804268</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B209" s="3" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="C209" s="3" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="D209" s="3" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="E209" s="4" t="n">
+        <v>0.0881863560732114</v>
+      </c>
+      <c r="F209" s="4" t="n">
+        <v>0.102446483180428</v>
+      </c>
+      <c r="G209" s="4" t="n">
+        <v>0.0952932124768404</v>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B210" s="3" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="C210" s="3" t="n">
+        <v>18.67</v>
+      </c>
+      <c r="E210" s="4" t="n">
+        <v>0.0924517261556467</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B211" s="3" t="n">
+        <v>-0.79</v>
+      </c>
+      <c r="C211" s="3" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="D211" s="3" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="E211" s="4" t="n">
+        <v>13.1392405063291</v>
+      </c>
+      <c r="F211" s="4" t="n">
+        <v>0.0802919708029197</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B212" s="3" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="C212" s="3" t="n">
+        <v>8.27</v>
+      </c>
+      <c r="D212" s="3" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="E212" s="4" t="n">
+        <v>0.140689655172414</v>
+      </c>
+      <c r="F212" s="4" t="n">
+        <v>0.129383313180169</v>
+      </c>
+      <c r="G212" s="4" t="n">
+        <v>0.135022405976625</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B213" s="3" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="C213" s="3" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="D213" s="3" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="E213" s="4" t="n">
+        <v>-0.0456730769230769</v>
+      </c>
+      <c r="F213" s="4" t="n">
+        <v>-0.123425692695214</v>
+      </c>
+      <c r="G213" s="4" t="n">
+        <v>-0.0853752345696835</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B214" s="3" t="n">
+        <v>44.27</v>
+      </c>
+      <c r="C214" s="3" t="n">
+        <v>50.33</v>
+      </c>
+      <c r="D214" s="3" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="E214" s="4" t="n">
+        <v>0.136887282584143</v>
+      </c>
+      <c r="F214" s="4" t="n">
+        <v>0.140274190343731</v>
+      </c>
+      <c r="G214" s="4" t="n">
+        <v>0.138579477094471</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B215" s="3" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="C215" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="D215" s="3" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="E215" s="4" t="n">
+        <v>2.96551724137931</v>
+      </c>
+      <c r="F215" s="4" t="n">
+        <v>0.539130434782609</v>
+      </c>
+      <c r="G215" s="4" t="n">
+        <v>1.47051579146179</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B216" s="3" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="C216" s="3" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="D216" s="3" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="E216" s="4" t="n">
+        <v>2.48905109489051</v>
+      </c>
+      <c r="F216" s="4" t="n">
+        <v>0.141213389121339</v>
+      </c>
+      <c r="G216" s="4" t="n">
+        <v>0.995432741241237</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B217" s="3" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="C217" s="3" t="n">
+        <v>16.09</v>
+      </c>
+      <c r="D217" s="3" t="n">
+        <v>16.93</v>
+      </c>
+      <c r="E217" s="4" t="n">
+        <v>0.0755347593582887</v>
+      </c>
+      <c r="F217" s="4" t="n">
+        <v>0.0522063393412057</v>
+      </c>
+      <c r="G217" s="4" t="n">
+        <v>0.0638066045943735</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B218" s="3" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="C218" s="3" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="D218" s="3" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="E218" s="4" t="n">
+        <v>0.0970350404312668</v>
+      </c>
+      <c r="F218" s="4" t="n">
+        <v>0.0786240786240785</v>
+      </c>
+      <c r="G218" s="4" t="n">
+        <v>0.0877906093102219</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B219" s="3" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="C219" s="3" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="D219" s="3" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="E219" s="4" t="n">
+        <v>-0.00938967136150236</v>
+      </c>
+      <c r="F219" s="4" t="n">
+        <v>-0.0331753554502369</v>
+      </c>
+      <c r="G219" s="4" t="n">
+        <v>-0.0213547737442136</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B220" s="3" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="C220" s="3" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="D220" s="3" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E220" s="4" t="n">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="F220" s="4" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B221" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C221" s="3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D221" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E221" s="4" t="n">
+        <v>0.344827586206897</v>
+      </c>
+      <c r="F221" s="4" t="n">
+        <v>0.269230769230769</v>
+      </c>
+      <c r="G221" s="4" t="n">
+        <v>0.306482511067078</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B222" s="3" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="C222" s="3" t="n">
+        <v>13.32</v>
+      </c>
+      <c r="D222" s="3" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="E222" s="4" t="n">
+        <v>0.160278745644599</v>
+      </c>
+      <c r="F222" s="4" t="n">
+        <v>0.144144144144144</v>
+      </c>
+      <c r="G222" s="4" t="n">
+        <v>0.152183202621953</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B223" s="3" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="C223" s="3" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D223" s="3" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="E223" s="4" t="n">
+        <v>0.63594470046083</v>
+      </c>
+      <c r="F223" s="4" t="n">
+        <v>0.391549295774648</v>
+      </c>
+      <c r="G223" s="4" t="n">
+        <v>0.5088067125555</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B224" s="3" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="C224" s="3" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="D224" s="3" t="n">
+        <v>8.05</v>
+      </c>
+      <c r="E224" s="4" t="n">
+        <v>0.187376725838264</v>
+      </c>
+      <c r="F224" s="4" t="n">
+        <v>0.337209302325582</v>
+      </c>
+      <c r="G224" s="4" t="n">
+        <v>0.260067935928781</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B225" s="3" t="n">
+        <v>18.39</v>
+      </c>
+      <c r="C225" s="3" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="D225" s="3" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="E225" s="4" t="n">
+        <v>0.136487221315932</v>
+      </c>
+      <c r="F225" s="4" t="n">
+        <v>0.174641148325359</v>
+      </c>
+      <c r="G225" s="4" t="n">
+        <v>0.155406705322262</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B226" s="3" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="C226" s="3" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="D226" s="3" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="E226" s="4" t="n">
+        <v>-0.08955223880597</v>
+      </c>
+      <c r="F226" s="4" t="n">
+        <v>-0.0491803278688525</v>
+      </c>
+      <c r="G226" s="4" t="n">
+        <v>-0.0695852313129134</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G197"/>
+  <autoFilter ref="A1:G226"/>
   <conditionalFormatting sqref="E2:E197">
     <cfRule type="colorScale" priority="2">
       <colorScale>

</xml_diff>